<commit_message>
Guestpay and VT Sale Transactions test case
</commit_message>
<xml_diff>
--- a/TestData/GuestPaymentData.xlsx
+++ b/TestData/GuestPaymentData.xlsx
@@ -92,7 +92,7 @@
     <x:t>Pass</x:t>
   </x:si>
   <x:si>
-    <x:t>07/24/2024 19:16:24</x:t>
+    <x:t>11/19/2024 20:28:40</x:t>
   </x:si>
   <x:si>
     <x:t>Y</x:t>
@@ -119,7 +119,7 @@
     <x:t>Two transactions in the amount of $10.00 and $1.00 will appear on your Credit Card or Bank statement</x:t>
   </x:si>
   <x:si>
-    <x:t>07/24/2024 19:17:26</x:t>
+    <x:t>11/19/2024 20:29:13</x:t>
   </x:si>
   <x:si>
     <x:t>Ayesha Kowkab</x:t>
@@ -564,7 +564,7 @@
     <x:pageSetUpPr fitToPage="false"/>
   </x:sheetPr>
   <x:dimension ref="A1:V3"/>
-  <x:sheetFormatPr defaultColWidth="52.767031" defaultRowHeight="12.8" zeroHeight="false"/>
+  <x:sheetFormatPr defaultColWidth="78.349531" defaultRowHeight="12.8" zeroHeight="false"/>
   <x:sheetData>
     <x:row r="1" spans="1:22" customFormat="1" ht="13" customHeight="1" outlineLevel="0">
       <x:c r="A1" s="1" t="s">

</xml_diff>